<commit_message>
Assessed a different development classification
</commit_message>
<xml_diff>
--- a/Copper/1. Running BLM/Data inputs/BLM_Data_Entry_for_Cu.xlsx
+++ b/Copper/1. Running BLM/Data inputs/BLM_Data_Entry_for_Cu.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://ornl-my.sharepoint.com/personal/q4q_ornl_gov/Documents/Research/Bioavailability Project/BLM_spatial_assessmt/Copper/1. Running BLM/Data inputs/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="13" documentId="11_09D4BCDF8F79A8D366075C52F37BD2722A4C017D" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{66C98C88-2DF4-4638-86CD-CA06301CCA3D}"/>
+  <xr:revisionPtr revIDLastSave="16" documentId="11_09D4BCDF8F79A8D366075C52F37BD2722A4C017D" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{EEE040C8-D8B9-4809-9166-E05D0A33D24D}"/>
   <bookViews>
-    <workbookView xWindow="21960" yWindow="3290" windowWidth="16390" windowHeight="15370" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="23440" yWindow="5510" windowWidth="28800" windowHeight="15370" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -1715,6 +1715,9 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:O387"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="10.1796875" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:15" s="1" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
@@ -1783,7 +1786,7 @@
         <v>0.91071829999999998</v>
       </c>
       <c r="G2">
-        <v>70</v>
+        <v>10</v>
       </c>
       <c r="H2">
         <v>60.036844000000002</v>
@@ -1830,7 +1833,7 @@
         <v>1.9216</v>
       </c>
       <c r="G3">
-        <v>70</v>
+        <v>10</v>
       </c>
       <c r="H3">
         <v>53.624364</v>
@@ -1877,7 +1880,7 @@
         <v>0.43031829999999999</v>
       </c>
       <c r="G4">
-        <v>70</v>
+        <v>10</v>
       </c>
       <c r="H4">
         <v>10.861138</v>
@@ -1924,7 +1927,7 @@
         <v>6.3352750000000002</v>
       </c>
       <c r="G5">
-        <v>70</v>
+        <v>10</v>
       </c>
       <c r="H5">
         <v>12.263868</v>
@@ -1971,7 +1974,7 @@
         <v>1.4312317000000001</v>
       </c>
       <c r="G6">
-        <v>70</v>
+        <v>10</v>
       </c>
       <c r="H6">
         <v>6.5727920000000006</v>
@@ -2018,7 +2021,7 @@
         <v>0.98085670000000003</v>
       </c>
       <c r="G7">
-        <v>70</v>
+        <v>10</v>
       </c>
       <c r="H7">
         <v>1.843588</v>
@@ -2065,7 +2068,7 @@
         <v>1.0709317</v>
       </c>
       <c r="G8">
-        <v>70</v>
+        <v>10</v>
       </c>
       <c r="H8">
         <v>16.792681999999999</v>
@@ -2112,7 +2115,7 @@
         <v>1.1309817</v>
       </c>
       <c r="G9">
-        <v>70</v>
+        <v>10</v>
       </c>
       <c r="H9">
         <v>53.664442000000001</v>
@@ -2159,7 +2162,7 @@
         <v>1.0809</v>
       </c>
       <c r="G10">
-        <v>70</v>
+        <v>10</v>
       </c>
       <c r="H10">
         <v>30.098578</v>
@@ -2206,7 +2209,7 @@
         <v>1.471225</v>
       </c>
       <c r="G11">
-        <v>70</v>
+        <v>10</v>
       </c>
       <c r="H11">
         <v>62.922460000000001</v>
@@ -2253,7 +2256,7 @@
         <v>1.1709750000000001</v>
       </c>
       <c r="G12">
-        <v>70</v>
+        <v>10</v>
       </c>
       <c r="H12">
         <v>22.563914</v>
@@ -2300,7 +2303,7 @@
         <v>0.73056829999999995</v>
       </c>
       <c r="G13">
-        <v>70</v>
+        <v>10</v>
       </c>
       <c r="H13">
         <v>47.332118000000001</v>
@@ -2347,7 +2350,7 @@
         <v>1.3411567</v>
       </c>
       <c r="G14">
-        <v>70</v>
+        <v>10</v>
       </c>
       <c r="H14">
         <v>21.682198</v>
@@ -2394,7 +2397,7 @@
         <v>0.88069330000000001</v>
       </c>
       <c r="G15">
-        <v>70</v>
+        <v>10</v>
       </c>
       <c r="H15">
         <v>14.42808</v>
@@ -2441,7 +2444,7 @@
         <v>1.231025</v>
       </c>
       <c r="G16">
-        <v>70</v>
+        <v>10</v>
       </c>
       <c r="H16">
         <v>69.735720000000001</v>
@@ -2488,7 +2491,7 @@
         <v>1.2409933</v>
       </c>
       <c r="G17">
-        <v>70</v>
+        <v>10</v>
       </c>
       <c r="H17">
         <v>67.691742000000005</v>
@@ -2535,7 +2538,7 @@
         <v>1.0809</v>
       </c>
       <c r="G18">
-        <v>70</v>
+        <v>10</v>
       </c>
       <c r="H18">
         <v>63.243084000000003</v>
@@ -2582,7 +2585,7 @@
         <v>2.0417000000000001</v>
       </c>
       <c r="G19">
-        <v>70</v>
+        <v>10</v>
       </c>
       <c r="H19">
         <v>83.602708000000007</v>
@@ -2629,7 +2632,7 @@
         <v>1.0007933</v>
       </c>
       <c r="G20">
-        <v>70</v>
+        <v>10</v>
       </c>
       <c r="H20">
         <v>62.601836000000013</v>
@@ -2676,7 +2679,7 @@
         <v>1.7014567</v>
       </c>
       <c r="G21">
-        <v>70</v>
+        <v>10</v>
       </c>
       <c r="H21">
         <v>88.291834000000009</v>
@@ -2723,7 +2726,7 @@
         <v>0.96079999999999999</v>
       </c>
       <c r="G22">
-        <v>70</v>
+        <v>10</v>
       </c>
       <c r="H22">
         <v>56.469901999999998</v>
@@ -2770,7 +2773,7 @@
         <v>0.93077500000000002</v>
       </c>
       <c r="G23">
-        <v>70</v>
+        <v>10</v>
       </c>
       <c r="H23">
         <v>57.872632000000003</v>
@@ -2817,7 +2820,7 @@
         <v>0.75062499999999999</v>
       </c>
       <c r="G24">
-        <v>70</v>
+        <v>10</v>
       </c>
       <c r="H24">
         <v>56.750448000000013</v>
@@ -2864,7 +2867,7 @@
         <v>0.95083170000000006</v>
       </c>
       <c r="G25">
-        <v>70</v>
+        <v>10</v>
       </c>
       <c r="H25">
         <v>58.073022000000002</v>
@@ -2911,7 +2914,7 @@
         <v>2.4020000000000001</v>
       </c>
       <c r="G26">
-        <v>70</v>
+        <v>10</v>
       </c>
       <c r="H26">
         <v>86.768870000000007</v>
@@ -2958,7 +2961,7 @@
         <v>3.2927816999999999</v>
       </c>
       <c r="G27">
-        <v>70</v>
+        <v>10</v>
       </c>
       <c r="H27">
         <v>76.188278000000011</v>
@@ -3005,7 +3008,7 @@
         <v>2.5020433</v>
       </c>
       <c r="G28">
-        <v>70</v>
+        <v>10</v>
       </c>
       <c r="H28">
         <v>28.695848000000002</v>
@@ -3052,7 +3055,7 @@
         <v>1.7714749999999999</v>
       </c>
       <c r="G29">
-        <v>70</v>
+        <v>10</v>
       </c>
       <c r="H29">
         <v>66.569558000000001</v>
@@ -3099,7 +3102,7 @@
         <v>1.5712683000000001</v>
       </c>
       <c r="G30">
-        <v>70</v>
+        <v>10</v>
       </c>
       <c r="H30">
         <v>62.722070000000002</v>
@@ -3146,7 +3149,7 @@
         <v>2.2419066999999999</v>
       </c>
       <c r="G31">
-        <v>70</v>
+        <v>10</v>
       </c>
       <c r="H31">
         <v>31.781853999999999</v>
@@ -3193,7 +3196,7 @@
         <v>3.1025432999999998</v>
       </c>
       <c r="G32">
-        <v>70</v>
+        <v>10</v>
       </c>
       <c r="H32">
         <v>56.389746000000002</v>
@@ -3240,7 +3243,7 @@
         <v>2.2118817000000002</v>
       </c>
       <c r="G33">
-        <v>70</v>
+        <v>10</v>
       </c>
       <c r="H33">
         <v>53.904910000000001</v>
@@ -3287,7 +3290,7 @@
         <v>2.1717683000000001</v>
       </c>
       <c r="G34">
-        <v>70</v>
+        <v>10</v>
       </c>
       <c r="H34">
         <v>43.644942</v>
@@ -3334,7 +3337,7 @@
         <v>1.8114683</v>
       </c>
       <c r="G35">
-        <v>70</v>
+        <v>10</v>
       </c>
       <c r="H35">
         <v>40.599013999999997</v>
@@ -3381,7 +3384,7 @@
         <v>2.4419933</v>
       </c>
       <c r="G36">
-        <v>70</v>
+        <v>10</v>
       </c>
       <c r="H36">
         <v>52.502180000000003</v>
@@ -3428,7 +3431,7 @@
         <v>2.94245</v>
       </c>
       <c r="G37">
-        <v>70</v>
+        <v>10</v>
       </c>
       <c r="H37">
         <v>52.341868000000012</v>
@@ -3475,7 +3478,7 @@
         <v>3.1426566999999999</v>
       </c>
       <c r="G38">
-        <v>70</v>
+        <v>10</v>
       </c>
       <c r="H38">
         <v>62.922460000000001</v>
@@ -3522,7 +3525,7 @@
         <v>2.4119682999999998</v>
       </c>
       <c r="G39">
-        <v>70</v>
+        <v>10</v>
       </c>
       <c r="H39">
         <v>53.343818000000013</v>
@@ -3569,7 +3572,7 @@
         <v>2.9223933</v>
       </c>
       <c r="G40">
-        <v>70</v>
+        <v>10</v>
       </c>
       <c r="H40">
         <v>53.303739999999998</v>
@@ -3616,7 +3619,7 @@
         <v>3.1025432999999998</v>
       </c>
       <c r="G41">
-        <v>70</v>
+        <v>10</v>
       </c>
       <c r="H41">
         <v>53.023193999999997</v>
@@ -3663,7 +3666,7 @@
         <v>0.93077500000000002</v>
       </c>
       <c r="G42">
-        <v>70</v>
+        <v>10</v>
       </c>
       <c r="H42">
         <v>16.512136000000002</v>
@@ -3710,7 +3713,7 @@
         <v>2.6421999999999999</v>
       </c>
       <c r="G43">
-        <v>70</v>
+        <v>10</v>
       </c>
       <c r="H43">
         <v>54.786626000000012</v>
@@ -3757,7 +3760,7 @@
         <v>3.7630933</v>
       </c>
       <c r="G44">
-        <v>70</v>
+        <v>10</v>
       </c>
       <c r="H44">
         <v>18.716425999999998</v>
@@ -3804,7 +3807,7 @@
         <v>3.8131750000000002</v>
       </c>
       <c r="G45">
-        <v>70</v>
+        <v>10</v>
       </c>
       <c r="H45">
         <v>55.508030000000012</v>
@@ -3851,7 +3854,7 @@
         <v>3.8431999999999999</v>
       </c>
       <c r="G46">
-        <v>70</v>
+        <v>10</v>
       </c>
       <c r="H46">
         <v>46.370246000000002</v>
@@ -3898,7 +3901,7 @@
         <v>4.1534182999999993</v>
       </c>
       <c r="G47">
-        <v>70</v>
+        <v>10</v>
       </c>
       <c r="H47">
         <v>31.661619999999999</v>
@@ -3945,7 +3948,7 @@
         <v>3.5429499999999998</v>
       </c>
       <c r="G48">
-        <v>70</v>
+        <v>10</v>
       </c>
       <c r="H48">
         <v>27.65382</v>
@@ -3992,7 +3995,7 @@
         <v>4.0734317000000004</v>
       </c>
       <c r="G49">
-        <v>70</v>
+        <v>10</v>
       </c>
       <c r="H49">
         <v>36.350746000000001</v>
@@ -4039,7 +4042,7 @@
         <v>4.1134250000000003</v>
       </c>
       <c r="G50">
-        <v>70</v>
+        <v>10</v>
       </c>
       <c r="H50">
         <v>40.078000000000003</v>
@@ -4086,7 +4089,7 @@
         <v>4.2335250000000002</v>
       </c>
       <c r="G51">
-        <v>70</v>
+        <v>10</v>
       </c>
       <c r="H51">
         <v>43.845332000000013</v>
@@ -4133,7 +4136,7 @@
         <v>2.6322317000000002</v>
       </c>
       <c r="G52">
-        <v>70</v>
+        <v>10</v>
       </c>
       <c r="H52">
         <v>30.298967999999999</v>
@@ -4180,7 +4183,7 @@
         <v>2.4720182999999998</v>
       </c>
       <c r="G53">
-        <v>70</v>
+        <v>10</v>
       </c>
       <c r="H53">
         <v>22.523835999999999</v>
@@ -4227,7 +4230,7 @@
         <v>3.7030433</v>
       </c>
       <c r="G54">
-        <v>70</v>
+        <v>10</v>
       </c>
       <c r="H54">
         <v>29.056550000000001</v>
@@ -4274,7 +4277,7 @@
         <v>4.0734317000000004</v>
       </c>
       <c r="G55">
-        <v>70</v>
+        <v>10</v>
       </c>
       <c r="H55">
         <v>35.068249999999999</v>
@@ -4321,7 +4324,7 @@
         <v>4.3436567000000004</v>
       </c>
       <c r="G56">
-        <v>70</v>
+        <v>10</v>
       </c>
       <c r="H56">
         <v>37.553086</v>
@@ -4368,7 +4371,7 @@
         <v>4.0032933000000002</v>
       </c>
       <c r="G57">
-        <v>70</v>
+        <v>10</v>
       </c>
       <c r="H57">
         <v>34.226612000000003</v>
@@ -4415,7 +4418,7 @@
         <v>3.7231000000000001</v>
       </c>
       <c r="G58">
-        <v>70</v>
+        <v>10</v>
       </c>
       <c r="H58">
         <v>52.742648000000003</v>
@@ -4462,7 +4465,7 @@
         <v>5.1843567000000004</v>
       </c>
       <c r="G59">
-        <v>70</v>
+        <v>10</v>
       </c>
       <c r="H59">
         <v>63.323240000000013</v>
@@ -4509,7 +4512,7 @@
         <v>4.3035432999999994</v>
       </c>
       <c r="G60">
-        <v>70</v>
+        <v>10</v>
       </c>
       <c r="H60">
         <v>57.752398000000007</v>
@@ -4556,7 +4559,7 @@
         <v>8.7673000000000005</v>
       </c>
       <c r="G61">
-        <v>70</v>
+        <v>10</v>
       </c>
       <c r="H61">
         <v>17.954944000000001</v>
@@ -4603,7 +4606,7 @@
         <v>4.6538750000000002</v>
       </c>
       <c r="G62">
-        <v>70</v>
+        <v>10</v>
       </c>
       <c r="H62">
         <v>48.694770000000013</v>
@@ -4650,7 +4653,7 @@
         <v>4.6037933000000004</v>
       </c>
       <c r="G63">
-        <v>70</v>
+        <v>10</v>
       </c>
       <c r="H63">
         <v>49.897109999999998</v>
@@ -4697,7 +4700,7 @@
         <v>8.4570816999999998</v>
       </c>
       <c r="G64">
-        <v>70</v>
+        <v>10</v>
       </c>
       <c r="H64">
         <v>15.590342</v>
@@ -4744,7 +4747,7 @@
         <v>1.6613433</v>
       </c>
       <c r="G65">
-        <v>70</v>
+        <v>10</v>
       </c>
       <c r="H65">
         <v>62.802225999999997</v>
@@ -4791,7 +4794,7 @@
         <v>1.4312317000000001</v>
       </c>
       <c r="G66">
-        <v>70</v>
+        <v>10</v>
       </c>
       <c r="H66">
         <v>50.137577999999998</v>
@@ -4838,7 +4841,7 @@
         <v>1.6814</v>
       </c>
       <c r="G67">
-        <v>70</v>
+        <v>10</v>
       </c>
       <c r="H67">
         <v>56.830604000000001</v>
@@ -4885,7 +4888,7 @@
         <v>2.5821499999999999</v>
       </c>
       <c r="G68">
-        <v>70</v>
+        <v>10</v>
       </c>
       <c r="H68">
         <v>60.116999999999997</v>
@@ -4932,7 +4935,7 @@
         <v>1.7414499999999999</v>
       </c>
       <c r="G69">
-        <v>70</v>
+        <v>10</v>
       </c>
       <c r="H69">
         <v>55.347718</v>
@@ -4979,7 +4982,7 @@
         <v>3.4128816999999998</v>
       </c>
       <c r="G70">
-        <v>70</v>
+        <v>10</v>
       </c>
       <c r="H70">
         <v>70.136499999999998</v>
@@ -5026,7 +5029,7 @@
         <v>3.0124683000000001</v>
       </c>
       <c r="G71">
-        <v>70</v>
+        <v>10</v>
       </c>
       <c r="H71">
         <v>40.999794000000001</v>
@@ -5073,7 +5076,7 @@
         <v>3.4027932999999999</v>
       </c>
       <c r="G72">
-        <v>70</v>
+        <v>10</v>
       </c>
       <c r="H72">
         <v>25.449529999999999</v>
@@ -5120,7 +5123,7 @@
         <v>2.4620500000000001</v>
       </c>
       <c r="G73">
-        <v>70</v>
+        <v>10</v>
       </c>
       <c r="H73">
         <v>14.62847</v>
@@ -5167,7 +5170,7 @@
         <v>2.3719749999999999</v>
       </c>
       <c r="G74">
-        <v>70</v>
+        <v>10</v>
       </c>
       <c r="H74">
         <v>18.395802</v>
@@ -5214,7 +5217,7 @@
         <v>1.6913682999999999</v>
       </c>
       <c r="G75">
-        <v>70</v>
+        <v>10</v>
       </c>
       <c r="H75">
         <v>1.8836660000000001</v>
@@ -5261,7 +5264,7 @@
         <v>1.6613433</v>
       </c>
       <c r="G76">
-        <v>70</v>
+        <v>10</v>
       </c>
       <c r="H76">
         <v>5.6910760000000007</v>
@@ -5308,7 +5311,7 @@
         <v>1.8515817000000001</v>
       </c>
       <c r="G77">
-        <v>70</v>
+        <v>10</v>
       </c>
       <c r="H77">
         <v>18.676348000000001</v>
@@ -5355,7 +5358,7 @@
         <v>2.4720182999999998</v>
       </c>
       <c r="G78">
-        <v>70</v>
+        <v>10</v>
       </c>
       <c r="H78">
         <v>27.693898000000001</v>
@@ -5402,7 +5405,7 @@
         <v>2.6421999999999999</v>
       </c>
       <c r="G79">
-        <v>70</v>
+        <v>10</v>
       </c>
       <c r="H79">
         <v>42.763226000000003</v>
@@ -5449,7 +5452,7 @@
         <v>0.5804433</v>
       </c>
       <c r="G80">
-        <v>70</v>
+        <v>10</v>
       </c>
       <c r="H80">
         <v>9.298096000000001</v>
@@ -5496,7 +5499,7 @@
         <v>8.2568749999999991</v>
       </c>
       <c r="G81">
-        <v>70</v>
+        <v>10</v>
       </c>
       <c r="H81">
         <v>13.866987999999999</v>
@@ -5543,7 +5546,7 @@
         <v>1.3610933000000001</v>
       </c>
       <c r="G82">
-        <v>70</v>
+        <v>10</v>
       </c>
       <c r="H82">
         <v>50.538358000000002</v>
@@ -5590,7 +5593,7 @@
         <v>4.9141317000000004</v>
       </c>
       <c r="G83">
-        <v>70</v>
+        <v>10</v>
       </c>
       <c r="H83">
         <v>64.285111999999998</v>
@@ -5637,7 +5640,7 @@
         <v>1.86155</v>
       </c>
       <c r="G84">
-        <v>70</v>
+        <v>10</v>
       </c>
       <c r="H84">
         <v>41.520808000000002</v>
@@ -5684,7 +5687,7 @@
         <v>1.0809</v>
       </c>
       <c r="G85">
-        <v>70</v>
+        <v>10</v>
       </c>
       <c r="H85">
         <v>8.6568480000000001</v>
@@ -5731,7 +5734,7 @@
         <v>3.4462695000000001</v>
       </c>
       <c r="G86">
-        <v>70</v>
+        <v>10</v>
       </c>
       <c r="H86">
         <v>48.49438</v>
@@ -5778,7 +5781,7 @@
         <v>1.1880291999999999</v>
       </c>
       <c r="G87">
-        <v>70</v>
+        <v>10</v>
       </c>
       <c r="H87">
         <v>53.303739999999998</v>
@@ -5825,7 +5828,7 @@
         <v>3.1108302000000001</v>
       </c>
       <c r="G88">
-        <v>70</v>
+        <v>10</v>
       </c>
       <c r="H88">
         <v>48.213834000000013</v>
@@ -5872,7 +5875,7 @@
         <v>3.0617093</v>
       </c>
       <c r="G89">
-        <v>70</v>
+        <v>10</v>
       </c>
       <c r="H89">
         <v>50.458202</v>
@@ -5919,7 +5922,7 @@
         <v>3.5810217</v>
       </c>
       <c r="G90">
-        <v>70</v>
+        <v>10</v>
       </c>
       <c r="H90">
         <v>48.975316000000007</v>
@@ -5966,7 +5969,7 @@
         <v>4.4128343000000001</v>
       </c>
       <c r="G91">
-        <v>70</v>
+        <v>10</v>
       </c>
       <c r="H91">
         <v>52.90296</v>
@@ -6013,7 +6016,7 @@
         <v>2.0093931</v>
       </c>
       <c r="G92">
-        <v>70</v>
+        <v>10</v>
       </c>
       <c r="H92">
         <v>52.542257999999997</v>
@@ -6060,7 +6063,7 @@
         <v>2.8432474000000001</v>
       </c>
       <c r="G93">
-        <v>70</v>
+        <v>10</v>
       </c>
       <c r="H93">
         <v>55.708419999999997</v>
@@ -6107,7 +6110,7 @@
         <v>1.6614633999999999</v>
       </c>
       <c r="G94">
-        <v>70</v>
+        <v>10</v>
       </c>
       <c r="H94">
         <v>46.330168</v>
@@ -6154,7 +6157,7 @@
         <v>1.8306842999999999</v>
       </c>
       <c r="G95">
-        <v>70</v>
+        <v>10</v>
       </c>
       <c r="H95">
         <v>53.383896</v>
@@ -6201,7 +6204,7 @@
         <v>2.1003088000000001</v>
       </c>
       <c r="G96">
-        <v>70</v>
+        <v>10</v>
       </c>
       <c r="H96">
         <v>55.067172000000006</v>
@@ -6248,7 +6251,7 @@
         <v>1.6060973000000001</v>
       </c>
       <c r="G97">
-        <v>70</v>
+        <v>10</v>
       </c>
       <c r="H97">
         <v>52.181556</v>
@@ -6295,7 +6298,7 @@
         <v>1.1682127</v>
       </c>
       <c r="G98">
-        <v>70</v>
+        <v>10</v>
       </c>
       <c r="H98">
         <v>54.626314000000001</v>
@@ -6342,7 +6345,7 @@
         <v>2.0073514000000001</v>
       </c>
       <c r="G99">
-        <v>70</v>
+        <v>10</v>
       </c>
       <c r="H99">
         <v>56.950837999999997</v>
@@ -6389,7 +6392,7 @@
         <v>1.5089364000000001</v>
       </c>
       <c r="G100">
-        <v>70</v>
+        <v>10</v>
       </c>
       <c r="H100">
         <v>44.446502000000002</v>
@@ -6436,7 +6439,7 @@
         <v>0.69261669999999997</v>
       </c>
       <c r="G101">
-        <v>70</v>
+        <v>10</v>
       </c>
       <c r="H101">
         <v>49.215784000000014</v>
@@ -6483,7 +6486,7 @@
         <v>1.5349980999999999</v>
       </c>
       <c r="G102">
-        <v>70</v>
+        <v>10</v>
       </c>
       <c r="H102">
         <v>76.949759999999998</v>
@@ -6530,7 +6533,7 @@
         <v>0.73429140000000004</v>
       </c>
       <c r="G103">
-        <v>70</v>
+        <v>10</v>
       </c>
       <c r="H103">
         <v>53.624364</v>
@@ -6577,7 +6580,7 @@
         <v>0.30085050000000002</v>
       </c>
       <c r="G104">
-        <v>70</v>
+        <v>10</v>
       </c>
       <c r="H104">
         <v>46.450401999999997</v>
@@ -6624,7 +6627,7 @@
         <v>0.43356099999999997</v>
       </c>
       <c r="G105">
-        <v>70</v>
+        <v>10</v>
       </c>
       <c r="H105">
         <v>46.129778000000002</v>
@@ -6671,7 +6674,7 @@
         <v>0.9717290999999999</v>
       </c>
       <c r="G106">
-        <v>70</v>
+        <v>10</v>
       </c>
       <c r="H106">
         <v>67.491352000000006</v>
@@ -6718,7 +6721,7 @@
         <v>1.0272152999999999</v>
       </c>
       <c r="G107">
-        <v>70</v>
+        <v>10</v>
       </c>
       <c r="H107">
         <v>64.886282000000008</v>
@@ -6765,7 +6768,7 @@
         <v>0.54657509999999998</v>
       </c>
       <c r="G108">
-        <v>70</v>
+        <v>10</v>
       </c>
       <c r="H108">
         <v>48.213834000000013</v>
@@ -6812,7 +6815,7 @@
         <v>0.50514060000000005</v>
       </c>
       <c r="G109">
-        <v>70</v>
+        <v>10</v>
       </c>
       <c r="H109">
         <v>47.051572</v>
@@ -6859,7 +6862,7 @@
         <v>0.32823330000000001</v>
       </c>
       <c r="G110">
-        <v>70</v>
+        <v>10</v>
       </c>
       <c r="H110">
         <v>36.190434000000003</v>
@@ -6906,7 +6909,7 @@
         <v>1.0104013000000001</v>
       </c>
       <c r="G111">
-        <v>70</v>
+        <v>10</v>
       </c>
       <c r="H111">
         <v>55.988965999999998</v>
@@ -6953,7 +6956,7 @@
         <v>0.83589599999999997</v>
       </c>
       <c r="G112">
-        <v>70</v>
+        <v>10</v>
       </c>
       <c r="H112">
         <v>27.012571999999999</v>
@@ -7000,7 +7003,7 @@
         <v>0.8798526000000001</v>
       </c>
       <c r="G113">
-        <v>70</v>
+        <v>10</v>
       </c>
       <c r="H113">
         <v>63.243084000000003</v>
@@ -7047,7 +7050,7 @@
         <v>1.2455571000000001</v>
       </c>
       <c r="G114">
-        <v>70</v>
+        <v>10</v>
       </c>
       <c r="H114">
         <v>37.953865999999998</v>
@@ -7094,7 +7097,7 @@
         <v>1.9111513</v>
       </c>
       <c r="G115">
-        <v>70</v>
+        <v>10</v>
       </c>
       <c r="H115">
         <v>47.011494000000013</v>
@@ -7141,7 +7144,7 @@
         <v>0.48364269999999998</v>
       </c>
       <c r="G116">
-        <v>70</v>
+        <v>10</v>
       </c>
       <c r="H116">
         <v>48.694770000000013</v>
@@ -7188,7 +7191,7 @@
         <v>0.43512230000000002</v>
       </c>
       <c r="G117">
-        <v>70</v>
+        <v>10</v>
       </c>
       <c r="H117">
         <v>55.027094000000012</v>
@@ -7235,7 +7238,7 @@
         <v>2.1796948999999999</v>
       </c>
       <c r="G118">
-        <v>70</v>
+        <v>10</v>
       </c>
       <c r="H118">
         <v>54.506079999999997</v>
@@ -7282,7 +7285,7 @@
         <v>1.5674250999999999</v>
       </c>
       <c r="G119">
-        <v>70</v>
+        <v>10</v>
       </c>
       <c r="H119">
         <v>52.021244000000003</v>
@@ -7329,7 +7332,7 @@
         <v>3.1081880000000002</v>
       </c>
       <c r="G120">
-        <v>70</v>
+        <v>10</v>
       </c>
       <c r="H120">
         <v>54.185456000000002</v>
@@ -7376,7 +7379,7 @@
         <v>1.3771867</v>
       </c>
       <c r="G121">
-        <v>70</v>
+        <v>10</v>
       </c>
       <c r="H121">
         <v>47.572586000000001</v>
@@ -7423,7 +7426,7 @@
         <v>2.6698230000000001</v>
       </c>
       <c r="G122">
-        <v>70</v>
+        <v>10</v>
       </c>
       <c r="H122">
         <v>54.906860000000002</v>
@@ -7470,7 +7473,7 @@
         <v>1.2666947</v>
       </c>
       <c r="G123">
-        <v>70</v>
+        <v>10</v>
       </c>
       <c r="H123">
         <v>50.979216000000001</v>
@@ -7517,7 +7520,7 @@
         <v>2.8255927000000001</v>
       </c>
       <c r="G124">
-        <v>70</v>
+        <v>10</v>
       </c>
       <c r="H124">
         <v>57.952788000000012</v>
@@ -7564,7 +7567,7 @@
         <v>1.4306312000000001</v>
       </c>
       <c r="G125">
-        <v>70</v>
+        <v>10</v>
       </c>
       <c r="H125">
         <v>59.195206000000013</v>
@@ -7611,7 +7614,7 @@
         <v>1.2539640999999999</v>
       </c>
       <c r="G126">
-        <v>70</v>
+        <v>10</v>
       </c>
       <c r="H126">
         <v>46.370246000000002</v>
@@ -7658,7 +7661,7 @@
         <v>1.3836721000000001</v>
       </c>
       <c r="G127">
-        <v>70</v>
+        <v>10</v>
       </c>
       <c r="H127">
         <v>58.674192000000012</v>
@@ -7705,7 +7708,7 @@
         <v>1.3377939000000001</v>
       </c>
       <c r="G128">
-        <v>70</v>
+        <v>10</v>
       </c>
       <c r="H128">
         <v>55.948887999999997</v>
@@ -7752,7 +7755,7 @@
         <v>1.4043292999999999</v>
       </c>
       <c r="G129">
-        <v>70</v>
+        <v>10</v>
       </c>
       <c r="H129">
         <v>53.063271999999998</v>
@@ -7799,7 +7802,7 @@
         <v>0.71315380000000006</v>
       </c>
       <c r="G130">
-        <v>70</v>
+        <v>10</v>
       </c>
       <c r="H130">
         <v>53.544207999999998</v>
@@ -7846,7 +7849,7 @@
         <v>1.4061307999999999</v>
       </c>
       <c r="G131">
-        <v>70</v>
+        <v>10</v>
       </c>
       <c r="H131">
         <v>80.356390000000005</v>
@@ -7893,7 +7896,7 @@
         <v>0.90014950000000005</v>
       </c>
       <c r="G132">
-        <v>70</v>
+        <v>10</v>
       </c>
       <c r="H132">
         <v>60.678092000000007</v>
@@ -7940,7 +7943,7 @@
         <v>2.6506069999999999</v>
       </c>
       <c r="G133">
-        <v>70</v>
+        <v>10</v>
       </c>
       <c r="H133">
         <v>48.534458000000001</v>
@@ -7987,7 +7990,7 @@
         <v>2.3785805</v>
       </c>
       <c r="G134">
-        <v>70</v>
+        <v>10</v>
       </c>
       <c r="H134">
         <v>59.195206000000013</v>
@@ -8034,7 +8037,7 @@
         <v>0.67568260000000002</v>
       </c>
       <c r="G135">
-        <v>70</v>
+        <v>10</v>
       </c>
       <c r="H135">
         <v>54.025143999999997</v>
@@ -8081,7 +8084,7 @@
         <v>0.42251179999999999</v>
       </c>
       <c r="G136">
-        <v>70</v>
+        <v>10</v>
       </c>
       <c r="H136">
         <v>49.015394000000001</v>
@@ -8128,7 +8131,7 @@
         <v>0.59797789999999995</v>
       </c>
       <c r="G137">
-        <v>70</v>
+        <v>10</v>
       </c>
       <c r="H137">
         <v>48.694770000000013</v>
@@ -8175,7 +8178,7 @@
         <v>0.26734259999999999</v>
       </c>
       <c r="G138">
-        <v>70</v>
+        <v>10</v>
       </c>
       <c r="H138">
         <v>38.875660000000003</v>
@@ -8222,7 +8225,7 @@
         <v>3.0342064</v>
       </c>
       <c r="G139">
-        <v>70</v>
+        <v>10</v>
       </c>
       <c r="H139">
         <v>38.595114000000002</v>
@@ -8269,7 +8272,7 @@
         <v>0.66919719999999994</v>
       </c>
       <c r="G140">
-        <v>70</v>
+        <v>10</v>
       </c>
       <c r="H140">
         <v>57.391696000000003</v>
@@ -8316,7 +8319,7 @@
         <v>0.35225329999999999</v>
       </c>
       <c r="G141">
-        <v>70</v>
+        <v>10</v>
       </c>
       <c r="H141">
         <v>23.886488</v>
@@ -8363,7 +8366,7 @@
         <v>0.94602769999999992</v>
       </c>
       <c r="G142">
-        <v>70</v>
+        <v>10</v>
       </c>
       <c r="H142">
         <v>61.519730000000003</v>
@@ -8410,7 +8413,7 @@
         <v>1.0891869000000001</v>
       </c>
       <c r="G143">
-        <v>70</v>
+        <v>10</v>
       </c>
       <c r="H143">
         <v>29.978344</v>
@@ -8457,7 +8460,7 @@
         <v>0.87132549999999998</v>
       </c>
       <c r="G144">
-        <v>70</v>
+        <v>10</v>
       </c>
       <c r="H144">
         <v>34.627392</v>
@@ -8504,7 +8507,7 @@
         <v>1.9625541</v>
       </c>
       <c r="G145">
-        <v>70</v>
+        <v>10</v>
       </c>
       <c r="H145">
         <v>48.975316000000007</v>
@@ -8551,7 +8554,7 @@
         <v>1.6322791000000001</v>
       </c>
       <c r="G146">
-        <v>70</v>
+        <v>10</v>
       </c>
       <c r="H146">
         <v>47.732898000000013</v>
@@ -8598,7 +8601,7 @@
         <v>1.0739342000000001</v>
       </c>
       <c r="G147">
-        <v>70</v>
+        <v>10</v>
       </c>
       <c r="H147">
         <v>39.316518000000002</v>
@@ -8645,7 +8648,7 @@
         <v>1.7652298</v>
       </c>
       <c r="G148">
-        <v>70</v>
+        <v>10</v>
       </c>
       <c r="H148">
         <v>50.538358000000002</v>
@@ -8692,7 +8695,7 @@
         <v>0.95623620000000009</v>
       </c>
       <c r="G149">
-        <v>70</v>
+        <v>10</v>
       </c>
       <c r="H149">
         <v>32.142555999999999</v>
@@ -8739,7 +8742,7 @@
         <v>1.3870349</v>
       </c>
       <c r="G150">
-        <v>70</v>
+        <v>10</v>
       </c>
       <c r="H150">
         <v>33.184584000000001</v>
@@ -8786,7 +8789,7 @@
         <v>2.0485457</v>
       </c>
       <c r="G151">
-        <v>70</v>
+        <v>10</v>
       </c>
       <c r="H151">
         <v>52.381946000000013</v>
@@ -8833,7 +8836,7 @@
         <v>2.2865839000000001</v>
       </c>
       <c r="G152">
-        <v>70</v>
+        <v>10</v>
       </c>
       <c r="H152">
         <v>54.706470000000003</v>
@@ -8880,7 +8883,7 @@
         <v>1.1942744000000001</v>
       </c>
       <c r="G153">
-        <v>70</v>
+        <v>10</v>
       </c>
       <c r="H153">
         <v>53.383896</v>
@@ -8927,7 +8930,7 @@
         <v>1.0358624999999999</v>
       </c>
       <c r="G154">
-        <v>70</v>
+        <v>10</v>
       </c>
       <c r="H154">
         <v>30.018422000000001</v>
@@ -8974,7 +8977,7 @@
         <v>1.1807030999999999</v>
       </c>
       <c r="G155">
-        <v>70</v>
+        <v>10</v>
       </c>
       <c r="H155">
         <v>60.838403999999997</v>
@@ -9021,7 +9024,7 @@
         <v>1.1154888000000001</v>
       </c>
       <c r="G156">
-        <v>70</v>
+        <v>10</v>
       </c>
       <c r="H156">
         <v>56.229433999999998</v>
@@ -9068,7 +9071,7 @@
         <v>1.5779939000000001</v>
       </c>
       <c r="G157">
-        <v>70</v>
+        <v>10</v>
       </c>
       <c r="H157">
         <v>59.676142000000013</v>
@@ -9115,7 +9118,7 @@
         <v>0.96524370000000004</v>
       </c>
       <c r="G158">
-        <v>70</v>
+        <v>10</v>
       </c>
       <c r="H158">
         <v>49.49633</v>
@@ -9162,7 +9165,7 @@
         <v>1.6540172</v>
       </c>
       <c r="G159">
-        <v>70</v>
+        <v>10</v>
       </c>
       <c r="H159">
         <v>60.798326000000003</v>
@@ -9209,7 +9212,7 @@
         <v>0.4838829</v>
       </c>
       <c r="G160">
-        <v>70</v>
+        <v>10</v>
       </c>
       <c r="H160">
         <v>47.412273999999996</v>
@@ -9256,7 +9259,7 @@
         <v>0.99058480000000004</v>
       </c>
       <c r="G161">
-        <v>70</v>
+        <v>10</v>
       </c>
       <c r="H161">
         <v>84.92528200000001</v>
@@ -9303,7 +9306,7 @@
         <v>0.56519059999999999</v>
       </c>
       <c r="G162">
-        <v>70</v>
+        <v>10</v>
       </c>
       <c r="H162">
         <v>53.023193999999997</v>
@@ -9350,7 +9353,7 @@
         <v>2.1951877999999998</v>
       </c>
       <c r="G163">
-        <v>70</v>
+        <v>10</v>
       </c>
       <c r="H163">
         <v>75.106172000000001</v>
@@ -9397,7 +9400,7 @@
         <v>1.2150517000000001</v>
       </c>
       <c r="G164">
-        <v>70</v>
+        <v>10</v>
       </c>
       <c r="H164">
         <v>86.849026000000009</v>
@@ -9444,7 +9447,7 @@
         <v>0.37062859999999997</v>
       </c>
       <c r="G165">
-        <v>70</v>
+        <v>10</v>
       </c>
       <c r="H165">
         <v>42.001744000000002</v>
@@ -9491,7 +9494,7 @@
         <v>0.31886550000000002</v>
       </c>
       <c r="G166">
-        <v>70</v>
+        <v>10</v>
       </c>
       <c r="H166">
         <v>40.558936000000003</v>
@@ -9538,7 +9541,7 @@
         <v>0.39320739999999998</v>
       </c>
       <c r="G167">
-        <v>70</v>
+        <v>10</v>
       </c>
       <c r="H167">
         <v>43.644942</v>
@@ -9585,7 +9588,7 @@
         <v>1.0924296</v>
       </c>
       <c r="G168">
-        <v>70</v>
+        <v>10</v>
       </c>
       <c r="H168">
         <v>73.743520000000004</v>
@@ -9632,7 +9635,7 @@
         <v>0.47883870000000001</v>
       </c>
       <c r="G169">
-        <v>70</v>
+        <v>10</v>
       </c>
       <c r="H169">
         <v>46.811104</v>
@@ -9679,7 +9682,7 @@
         <v>0.54201129999999997</v>
       </c>
       <c r="G170">
-        <v>70</v>
+        <v>10</v>
       </c>
       <c r="H170">
         <v>43.364395999999999</v>
@@ -9726,7 +9729,7 @@
         <v>0.30589470000000002</v>
       </c>
       <c r="G171">
-        <v>70</v>
+        <v>10</v>
       </c>
       <c r="H171">
         <v>25.409452000000002</v>
@@ -9773,7 +9776,7 @@
         <v>1.086905</v>
       </c>
       <c r="G172">
-        <v>70</v>
+        <v>10</v>
       </c>
       <c r="H172">
         <v>6.2521680000000002</v>
@@ -9820,7 +9823,7 @@
         <v>1.9340904000000001</v>
       </c>
       <c r="G173">
-        <v>70</v>
+        <v>10</v>
       </c>
       <c r="H173">
         <v>52.542257999999997</v>
@@ -9867,7 +9870,7 @@
         <v>0.72444319999999995</v>
       </c>
       <c r="G174">
-        <v>70</v>
+        <v>10</v>
       </c>
       <c r="H174">
         <v>52.422024</v>
@@ -9914,7 +9917,7 @@
         <v>0.48628490000000002</v>
       </c>
       <c r="G175">
-        <v>70</v>
+        <v>10</v>
       </c>
       <c r="H175">
         <v>14.388002</v>
@@ -9961,7 +9964,7 @@
         <v>1.7904507999999999</v>
       </c>
       <c r="G176">
-        <v>70</v>
+        <v>10</v>
       </c>
       <c r="H176">
         <v>47.933287999999997</v>
@@ -10008,7 +10011,7 @@
         <v>1.7813232000000001</v>
       </c>
       <c r="G177">
-        <v>70</v>
+        <v>10</v>
       </c>
       <c r="H177">
         <v>19.558064000000002</v>
@@ -10055,7 +10058,7 @@
         <v>1.7213932999999999</v>
       </c>
       <c r="G178">
-        <v>70</v>
+        <v>10</v>
       </c>
       <c r="H178">
         <v>25.369374000000001</v>
@@ -10102,7 +10105,7 @@
         <v>1.1214938000000001</v>
       </c>
       <c r="G179">
-        <v>70</v>
+        <v>10</v>
       </c>
       <c r="H179">
         <v>9.3381740000000004</v>
@@ -10149,7 +10152,7 @@
         <v>1.4177805000000001</v>
       </c>
       <c r="G180">
-        <v>70</v>
+        <v>10</v>
       </c>
       <c r="H180">
         <v>2.4046799999999999</v>
@@ -10196,7 +10199,7 @@
         <v>0.56975439999999999</v>
       </c>
       <c r="G181">
-        <v>70</v>
+        <v>10</v>
       </c>
       <c r="H181">
         <v>45.969465999999997</v>
@@ -10243,7 +10246,7 @@
         <v>0.93425790000000009</v>
       </c>
       <c r="G182">
-        <v>70</v>
+        <v>10</v>
       </c>
       <c r="H182">
         <v>16.111356000000001</v>
@@ -10290,7 +10293,7 @@
         <v>2.5243818999999998</v>
       </c>
       <c r="G183">
-        <v>70</v>
+        <v>10</v>
       </c>
       <c r="H183">
         <v>50.337967999999996</v>
@@ -10337,7 +10340,7 @@
         <v>1.4792717</v>
       </c>
       <c r="G184">
-        <v>70</v>
+        <v>10</v>
       </c>
       <c r="H184">
         <v>44.246111999999997</v>
@@ -10384,7 +10387,7 @@
         <v>3.2260061000000002</v>
       </c>
       <c r="G185">
-        <v>70</v>
+        <v>10</v>
       </c>
       <c r="H185">
         <v>50.418124000000013</v>
@@ -10431,7 +10434,7 @@
         <v>3.3515106000000001</v>
       </c>
       <c r="G186">
-        <v>70</v>
+        <v>10</v>
       </c>
       <c r="H186">
         <v>50.017344000000001</v>
@@ -10478,7 +10481,7 @@
         <v>1.7518986999999999</v>
       </c>
       <c r="G187">
-        <v>70</v>
+        <v>10</v>
       </c>
       <c r="H187">
         <v>38.074100000000001</v>
@@ -10525,7 +10528,7 @@
         <v>1.5791949000000001</v>
       </c>
       <c r="G188">
-        <v>70</v>
+        <v>10</v>
       </c>
       <c r="H188">
         <v>37.352696000000002</v>
@@ -10572,7 +10575,7 @@
         <v>3.4886648</v>
       </c>
       <c r="G189">
-        <v>70</v>
+        <v>10</v>
       </c>
       <c r="H189">
         <v>51.860932000000012</v>
@@ -10619,7 +10622,7 @@
         <v>3.7214185999999998</v>
       </c>
       <c r="G190">
-        <v>70</v>
+        <v>10</v>
       </c>
       <c r="H190">
         <v>54.866782000000001</v>
@@ -10666,7 +10669,7 @@
         <v>1.8500204</v>
       </c>
       <c r="G191">
-        <v>70</v>
+        <v>10</v>
       </c>
       <c r="H191">
         <v>55.107250000000001</v>
@@ -10713,7 +10716,7 @@
         <v>1.7628277999999999</v>
       </c>
       <c r="G192">
-        <v>70</v>
+        <v>10</v>
       </c>
       <c r="H192">
         <v>35.629342000000001</v>
@@ -10760,7 +10763,7 @@
         <v>4.4648376000000001</v>
       </c>
       <c r="G193">
-        <v>70</v>
+        <v>10</v>
       </c>
       <c r="H193">
         <v>49.816954000000003</v>
@@ -10807,7 +10810,7 @@
         <v>1.9091096000000001</v>
       </c>
       <c r="G194">
-        <v>70</v>
+        <v>10</v>
       </c>
       <c r="H194">
         <v>61.479652000000002</v>
@@ -10854,7 +10857,7 @@
         <v>2.8370022000000001</v>
       </c>
       <c r="G195">
-        <v>70</v>
+        <v>10</v>
       </c>
       <c r="H195">
         <v>54.626314000000001</v>
@@ -10901,7 +10904,7 @@
         <v>5.7844964000000001</v>
       </c>
       <c r="G196">
-        <v>70</v>
+        <v>10</v>
       </c>
       <c r="H196">
         <v>32.182634</v>
@@ -10948,7 +10951,7 @@
         <v>1.7600655000000001</v>
       </c>
       <c r="G197">
-        <v>70</v>
+        <v>10</v>
       </c>
       <c r="H197">
         <v>57.231384000000013</v>
@@ -10995,7 +10998,7 @@
         <v>2.7743099999999998</v>
       </c>
       <c r="G198">
-        <v>70</v>
+        <v>10</v>
       </c>
       <c r="H198">
         <v>64.565657999999999</v>
@@ -11042,7 +11045,7 @@
         <v>5.2173841999999997</v>
       </c>
       <c r="G199">
-        <v>70</v>
+        <v>10</v>
       </c>
       <c r="H199">
         <v>84.92528200000001</v>
@@ -11089,7 +11092,7 @@
         <v>19.8922831</v>
       </c>
       <c r="G200">
-        <v>70</v>
+        <v>10</v>
       </c>
       <c r="H200">
         <v>18.556114000000001</v>
@@ -11136,7 +11139,7 @@
         <v>2.2907874000000001</v>
       </c>
       <c r="G201">
-        <v>70</v>
+        <v>10</v>
       </c>
       <c r="H201">
         <v>46.450401999999997</v>
@@ -11183,7 +11186,7 @@
         <v>18.274415999999999</v>
       </c>
       <c r="G202">
-        <v>70</v>
+        <v>10</v>
       </c>
       <c r="H202">
         <v>8.6568480000000001</v>
@@ -11230,7 +11233,7 @@
         <v>2.3453127999999999</v>
       </c>
       <c r="G203">
-        <v>70</v>
+        <v>10</v>
       </c>
       <c r="H203">
         <v>18.876738</v>
@@ -11277,7 +11280,7 @@
         <v>2.3208123999999999</v>
       </c>
       <c r="G204">
-        <v>70</v>
+        <v>10</v>
       </c>
       <c r="H204">
         <v>8.6969260000000013</v>
@@ -11324,7 +11327,7 @@
         <v>0.43644339999999998</v>
       </c>
       <c r="G205">
-        <v>70</v>
+        <v>10</v>
       </c>
       <c r="H205">
         <v>31.260840000000002</v>
@@ -11371,7 +11374,7 @@
         <v>1.8000588</v>
       </c>
       <c r="G206">
-        <v>70</v>
+        <v>10</v>
       </c>
       <c r="H206">
         <v>59.155127999999998</v>
@@ -11418,7 +11421,7 @@
         <v>1.7755584</v>
       </c>
       <c r="G207">
-        <v>70</v>
+        <v>10</v>
       </c>
       <c r="H207">
         <v>75.266484000000005</v>
@@ -11465,7 +11468,7 @@
         <v>14.2176782</v>
       </c>
       <c r="G208">
-        <v>70</v>
+        <v>10</v>
       </c>
       <c r="H208">
         <v>31.621542000000002</v>
@@ -11512,7 +11515,7 @@
         <v>4.2812047</v>
       </c>
       <c r="G209">
-        <v>70</v>
+        <v>10</v>
       </c>
       <c r="H209">
         <v>50.498280000000001</v>
@@ -11559,7 +11562,7 @@
         <v>6.1807062999999998</v>
       </c>
       <c r="G210">
-        <v>70</v>
+        <v>10</v>
       </c>
       <c r="H210">
         <v>40.118077999999997</v>
@@ -11606,7 +11609,7 @@
         <v>2.8234309</v>
       </c>
       <c r="G211">
-        <v>70</v>
+        <v>10</v>
       </c>
       <c r="H211">
         <v>26.932416</v>
@@ -11653,7 +11656,7 @@
         <v>1.5955284999999999</v>
       </c>
       <c r="G212">
-        <v>70</v>
+        <v>10</v>
       </c>
       <c r="H212">
         <v>2.4447580000000002</v>
@@ -11700,7 +11703,7 @@
         <v>1.889173</v>
       </c>
       <c r="G213">
-        <v>70</v>
+        <v>10</v>
       </c>
       <c r="H213">
         <v>29.777954000000001</v>
@@ -11747,7 +11750,7 @@
         <v>1.0984346</v>
       </c>
       <c r="G214">
-        <v>70</v>
+        <v>10</v>
       </c>
       <c r="H214">
         <v>18.435880000000001</v>
@@ -11794,7 +11797,7 @@
         <v>1.2865112000000001</v>
       </c>
       <c r="G215">
-        <v>70</v>
+        <v>10</v>
       </c>
       <c r="H215">
         <v>51.259762000000002</v>
@@ -11841,7 +11844,7 @@
         <v>3.4496323000000002</v>
       </c>
       <c r="G216">
-        <v>70</v>
+        <v>10</v>
       </c>
       <c r="H216">
         <v>26.291167999999999</v>
@@ -11888,7 +11891,7 @@
         <v>2.4935162000000002</v>
       </c>
       <c r="G217">
-        <v>70</v>
+        <v>10</v>
       </c>
       <c r="H217">
         <v>46.730948000000012</v>
@@ -11935,7 +11938,7 @@
         <v>1.8691163</v>
       </c>
       <c r="G218">
-        <v>70</v>
+        <v>10</v>
       </c>
       <c r="H218">
         <v>53.944988000000002</v>
@@ -11982,7 +11985,7 @@
         <v>7.1849825000000003</v>
       </c>
       <c r="G219">
-        <v>70</v>
+        <v>10</v>
       </c>
       <c r="H219">
         <v>28.695848000000002</v>
@@ -12029,7 +12032,7 @@
         <v>2.6891590999999999</v>
       </c>
       <c r="G220">
-        <v>70</v>
+        <v>10</v>
       </c>
       <c r="H220">
         <v>56.590136000000001</v>
@@ -12076,7 +12079,7 @@
         <v>1.7461339</v>
       </c>
       <c r="G221">
-        <v>70</v>
+        <v>10</v>
       </c>
       <c r="H221">
         <v>52.502180000000003</v>
@@ -12123,7 +12126,7 @@
         <v>3.2507467000000001</v>
       </c>
       <c r="G222">
-        <v>70</v>
+        <v>10</v>
       </c>
       <c r="H222">
         <v>57.151228000000003</v>
@@ -12170,7 +12173,7 @@
         <v>2.1437849999999998</v>
       </c>
       <c r="G223">
-        <v>70</v>
+        <v>10</v>
       </c>
       <c r="H223">
         <v>49.255862</v>
@@ -12217,7 +12220,7 @@
         <v>1.6338404</v>
       </c>
       <c r="G224">
-        <v>70</v>
+        <v>10</v>
       </c>
       <c r="H224">
         <v>45.488529999999997</v>
@@ -12264,7 +12267,7 @@
         <v>2.9717544</v>
       </c>
       <c r="G225">
-        <v>70</v>
+        <v>10</v>
       </c>
       <c r="H225">
         <v>53.744598000000003</v>
@@ -12311,7 +12314,7 @@
         <v>6.2126528999999993</v>
       </c>
       <c r="G226">
-        <v>70</v>
+        <v>10</v>
       </c>
       <c r="H226">
         <v>48.213834000000013</v>
@@ -12358,7 +12361,7 @@
         <v>8.026042799999999</v>
       </c>
       <c r="G227">
-        <v>70</v>
+        <v>10</v>
       </c>
       <c r="H227">
         <v>41.440652</v>
@@ -12405,7 +12408,7 @@
         <v>1.8683957</v>
       </c>
       <c r="G228">
-        <v>70</v>
+        <v>10</v>
       </c>
       <c r="H228">
         <v>43.083850000000012</v>
@@ -12452,7 +12455,7 @@
         <v>7.8983764999999986</v>
       </c>
       <c r="G229">
-        <v>70</v>
+        <v>10</v>
       </c>
       <c r="H229">
         <v>44.005643999999997</v>
@@ -12499,7 +12502,7 @@
         <v>6.0559224</v>
       </c>
       <c r="G230">
-        <v>70</v>
+        <v>10</v>
       </c>
       <c r="H230">
         <v>44.967516000000003</v>
@@ -12546,7 +12549,7 @@
         <v>2.8774758999999999</v>
       </c>
       <c r="G231">
-        <v>70</v>
+        <v>10</v>
       </c>
       <c r="H231">
         <v>60.758248000000002</v>
@@ -12593,7 +12596,7 @@
         <v>6.8866540999999986</v>
       </c>
       <c r="G232">
-        <v>70</v>
+        <v>10</v>
       </c>
       <c r="H232">
         <v>66.248934000000006</v>
@@ -12640,7 +12643,7 @@
         <v>4.6021118999999997</v>
       </c>
       <c r="G233">
-        <v>70</v>
+        <v>10</v>
       </c>
       <c r="H233">
         <v>68.533380000000008</v>
@@ -12687,7 +12690,7 @@
         <v>6.5215500999999998</v>
       </c>
       <c r="G234">
-        <v>70</v>
+        <v>10</v>
       </c>
       <c r="H234">
         <v>60.958638000000001</v>
@@ -12734,7 +12737,7 @@
         <v>5.6075891000000002</v>
       </c>
       <c r="G235">
-        <v>70</v>
+        <v>10</v>
       </c>
       <c r="H235">
         <v>56.870682000000002</v>
@@ -12781,7 +12784,7 @@
         <v>5.7380176999999994</v>
       </c>
       <c r="G236">
-        <v>70</v>
+        <v>10</v>
       </c>
       <c r="H236">
         <v>63.724020000000003</v>
@@ -12828,7 +12831,7 @@
         <v>5.8901843999999999</v>
       </c>
       <c r="G237">
-        <v>70</v>
+        <v>10</v>
       </c>
       <c r="H237">
         <v>48.895159999999997</v>
@@ -12875,7 +12878,7 @@
         <v>5.0641366000000003</v>
       </c>
       <c r="G238">
-        <v>70</v>
+        <v>10</v>
       </c>
       <c r="H238">
         <v>49.055472000000002</v>
@@ -12922,7 +12925,7 @@
         <v>0.49433159999999993</v>
       </c>
       <c r="G239">
-        <v>70</v>
+        <v>10</v>
       </c>
       <c r="H239">
         <v>51.420074000000007</v>
@@ -12969,7 +12972,7 @@
         <v>1.0116023000000001</v>
       </c>
       <c r="G240">
-        <v>70</v>
+        <v>10</v>
       </c>
       <c r="H240">
         <v>14.748704</v>
@@ -13016,7 +13019,7 @@
         <v>2.0550310999999999</v>
       </c>
       <c r="G241">
-        <v>70</v>
+        <v>10</v>
       </c>
       <c r="H241">
         <v>22.684148</v>
@@ -13063,7 +13066,7 @@
         <v>3.3947465999999999</v>
       </c>
       <c r="G242">
-        <v>70</v>
+        <v>10</v>
       </c>
       <c r="H242">
         <v>53.103350000000013</v>
@@ -13110,7 +13113,7 @@
         <v>1.8856900999999999</v>
       </c>
       <c r="G243">
-        <v>70</v>
+        <v>10</v>
       </c>
       <c r="H243">
         <v>60.878482000000012</v>
@@ -13157,7 +13160,7 @@
         <v>1.3620540999999999</v>
       </c>
       <c r="G244">
-        <v>70</v>
+        <v>10</v>
       </c>
       <c r="H244">
         <v>62.922460000000001</v>
@@ -13204,7 +13207,7 @@
         <v>0.94002269999999999</v>
       </c>
       <c r="G245">
-        <v>70</v>
+        <v>10</v>
       </c>
       <c r="H245">
         <v>52.702570000000001</v>
@@ -13251,7 +13254,7 @@
         <v>1.3195387000000001</v>
       </c>
       <c r="G246">
-        <v>70</v>
+        <v>10</v>
       </c>
       <c r="H246">
         <v>34.066300000000012</v>
@@ -13298,7 +13301,7 @@
         <v>0.74798280000000006</v>
       </c>
       <c r="G247">
-        <v>70</v>
+        <v>10</v>
       </c>
       <c r="H247">
         <v>37.673319999999997</v>
@@ -13345,7 +13348,7 @@
         <v>0.49325069999999999</v>
       </c>
       <c r="G248">
-        <v>70</v>
+        <v>10</v>
       </c>
       <c r="H248">
         <v>23.926566000000001</v>
@@ -13392,7 +13395,7 @@
         <v>1.2914353000000001</v>
       </c>
       <c r="G249">
-        <v>70</v>
+        <v>10</v>
       </c>
       <c r="H249">
         <v>58.313490000000002</v>
@@ -13439,7 +13442,7 @@
         <v>1.3919589999999999</v>
       </c>
       <c r="G250">
-        <v>70</v>
+        <v>10</v>
       </c>
       <c r="H250">
         <v>65.006516000000005</v>
@@ -13486,7 +13489,7 @@
         <v>2.5930791000000002</v>
       </c>
       <c r="G251">
-        <v>70</v>
+        <v>10</v>
       </c>
       <c r="H251">
         <v>70.897981999999999</v>
@@ -13533,7 +13536,7 @@
         <v>1.3241025</v>
       </c>
       <c r="G252">
-        <v>70</v>
+        <v>10</v>
       </c>
       <c r="H252">
         <v>60.397546000000013</v>
@@ -13580,7 +13583,7 @@
         <v>1.3032051</v>
       </c>
       <c r="G253">
-        <v>70</v>
+        <v>10</v>
       </c>
       <c r="H253">
         <v>58.674192000000012</v>
@@ -13627,7 +13630,7 @@
         <v>6.5396852000000001</v>
       </c>
       <c r="G254">
-        <v>70</v>
+        <v>10</v>
       </c>
       <c r="H254">
         <v>67.491352000000006</v>
@@ -13674,7 +13677,7 @@
         <v>5.1610573000000004</v>
       </c>
       <c r="G255">
-        <v>70</v>
+        <v>10</v>
       </c>
       <c r="H255">
         <v>49.175706000000012</v>
@@ -13721,7 +13724,7 @@
         <v>1.363135</v>
       </c>
       <c r="G256">
-        <v>70</v>
+        <v>10</v>
       </c>
       <c r="H256">
         <v>51.500230000000002</v>
@@ -13768,7 +13771,7 @@
         <v>2.7944868</v>
       </c>
       <c r="G257">
-        <v>70</v>
+        <v>10</v>
       </c>
       <c r="H257">
         <v>42.121978000000013</v>
@@ -13815,7 +13818,7 @@
         <v>3.4519142</v>
       </c>
       <c r="G258">
-        <v>70</v>
+        <v>10</v>
       </c>
       <c r="H258">
         <v>52.061321999999997</v>
@@ -13862,7 +13865,7 @@
         <v>1.363135</v>
       </c>
       <c r="G259">
-        <v>70</v>
+        <v>10</v>
       </c>
       <c r="H259">
         <v>55.588186</v>
@@ -13909,7 +13912,7 @@
         <v>1.5359589</v>
       </c>
       <c r="G260">
-        <v>70</v>
+        <v>10</v>
       </c>
       <c r="H260">
         <v>44.646892000000001</v>
@@ -13956,7 +13959,7 @@
         <v>3.5888282</v>
       </c>
       <c r="G261">
-        <v>70</v>
+        <v>10</v>
       </c>
       <c r="H261">
         <v>51.139528000000013</v>
@@ -14003,7 +14006,7 @@
         <v>3.0179928999999999</v>
       </c>
       <c r="G262">
-        <v>70</v>
+        <v>10</v>
       </c>
       <c r="H262">
         <v>50.939138</v>
@@ -14050,7 +14053,7 @@
         <v>3.4242911999999999</v>
       </c>
       <c r="G263">
-        <v>70</v>
+        <v>10</v>
       </c>
       <c r="H263">
         <v>55.067172000000006</v>
@@ -14097,7 +14100,7 @@
         <v>1.6076585999999999</v>
       </c>
       <c r="G264">
-        <v>70</v>
+        <v>10</v>
       </c>
       <c r="H264">
         <v>57.151228000000003</v>
@@ -14144,7 +14147,7 @@
         <v>1.3566495999999999</v>
       </c>
       <c r="G265">
-        <v>70</v>
+        <v>10</v>
       </c>
       <c r="H265">
         <v>46.570636</v>
@@ -14191,7 +14194,7 @@
         <v>1.5294734999999999</v>
       </c>
       <c r="G266">
-        <v>70</v>
+        <v>10</v>
       </c>
       <c r="H266">
         <v>55.748497999999998</v>
@@ -14238,7 +14241,7 @@
         <v>1.512059</v>
       </c>
       <c r="G267">
-        <v>70</v>
+        <v>10</v>
       </c>
       <c r="H267">
         <v>56.269512000000013</v>
@@ -14285,7 +14288,7 @@
         <v>2.3678916000000001</v>
       </c>
       <c r="G268">
-        <v>70</v>
+        <v>10</v>
       </c>
       <c r="H268">
         <v>58.073022000000002</v>
@@ -14332,7 +14335,7 @@
         <v>1.0495539</v>
       </c>
       <c r="G269">
-        <v>70</v>
+        <v>10</v>
       </c>
       <c r="H269">
         <v>62.241134000000002</v>
@@ -14379,7 +14382,7 @@
         <v>0.85006780000000004</v>
       </c>
       <c r="G270">
-        <v>70</v>
+        <v>10</v>
       </c>
       <c r="H270">
         <v>60.357467999999997</v>
@@ -14426,7 +14429,7 @@
         <v>1.512059</v>
       </c>
       <c r="G271">
-        <v>70</v>
+        <v>10</v>
       </c>
       <c r="H271">
         <v>78.392568000000011</v>
@@ -14473,7 +14476,7 @@
         <v>0.92825290000000005</v>
       </c>
       <c r="G272">
-        <v>70</v>
+        <v>10</v>
       </c>
       <c r="H272">
         <v>57.872632000000003</v>
@@ -14520,7 +14523,7 @@
         <v>1.0266147999999999</v>
       </c>
       <c r="G273">
-        <v>70</v>
+        <v>10</v>
       </c>
       <c r="H273">
         <v>80.79724800000001</v>
@@ -14567,7 +14570,7 @@
         <v>0.73345070000000001</v>
       </c>
       <c r="G274">
-        <v>70</v>
+        <v>10</v>
       </c>
       <c r="H274">
         <v>56.469901999999998</v>
@@ -14614,7 +14617,7 @@
         <v>0.68721219999999994</v>
       </c>
       <c r="G275">
-        <v>70</v>
+        <v>10</v>
       </c>
       <c r="H275">
         <v>54.786626000000012</v>
@@ -14661,7 +14664,7 @@
         <v>1.4771099000000001</v>
       </c>
       <c r="G276">
-        <v>70</v>
+        <v>10</v>
       </c>
       <c r="H276">
         <v>65.92831000000001</v>
@@ -14708,7 +14711,7 @@
         <v>0.3118997</v>
       </c>
       <c r="G277">
-        <v>70</v>
+        <v>10</v>
       </c>
       <c r="H277">
         <v>36.631292000000002</v>
@@ -14755,7 +14758,7 @@
         <v>0.64517720000000001</v>
       </c>
       <c r="G278">
-        <v>70</v>
+        <v>10</v>
       </c>
       <c r="H278">
         <v>54.425924000000002</v>
@@ -14802,7 +14805,7 @@
         <v>0.63532899999999992</v>
       </c>
       <c r="G279">
-        <v>70</v>
+        <v>10</v>
       </c>
       <c r="H279">
         <v>26.371324000000001</v>
@@ -14849,7 +14852,7 @@
         <v>0.96043970000000001</v>
       </c>
       <c r="G280">
-        <v>70</v>
+        <v>10</v>
       </c>
       <c r="H280">
         <v>74.224456000000004</v>
@@ -14896,7 +14899,7 @@
         <v>1.6600222</v>
       </c>
       <c r="G281">
-        <v>70</v>
+        <v>10</v>
       </c>
       <c r="H281">
         <v>42.322367999999997</v>
@@ -14943,7 +14946,7 @@
         <v>0.60410299999999995</v>
       </c>
       <c r="G282">
-        <v>70</v>
+        <v>10</v>
       </c>
       <c r="H282">
         <v>50.538358000000002</v>
@@ -14990,7 +14993,7 @@
         <v>1.1479158</v>
       </c>
       <c r="G283">
-        <v>70</v>
+        <v>10</v>
       </c>
       <c r="H283">
         <v>64.405346000000009</v>
@@ -15037,7 +15040,7 @@
         <v>1.6094600999999999</v>
       </c>
       <c r="G284">
-        <v>70</v>
+        <v>10</v>
       </c>
       <c r="H284">
         <v>55.988965999999998</v>
@@ -15084,7 +15087,7 @@
         <v>2.3805021000000002</v>
       </c>
       <c r="G285">
-        <v>70</v>
+        <v>10</v>
       </c>
       <c r="H285">
         <v>53.023193999999997</v>
@@ -15131,7 +15134,7 @@
         <v>3.0822463999999998</v>
       </c>
       <c r="G286">
-        <v>70</v>
+        <v>10</v>
       </c>
       <c r="H286">
         <v>50.899060000000013</v>
@@ -15178,7 +15181,7 @@
         <v>3.3946265000000002</v>
       </c>
       <c r="G287">
-        <v>70</v>
+        <v>10</v>
       </c>
       <c r="H287">
         <v>50.418124000000013</v>
@@ -15225,7 +15228,7 @@
         <v>3.3340961</v>
       </c>
       <c r="G288">
-        <v>70</v>
+        <v>10</v>
       </c>
       <c r="H288">
         <v>48.975316000000007</v>
@@ -15272,7 +15275,7 @@
         <v>2.9447318999999998</v>
       </c>
       <c r="G289">
-        <v>70</v>
+        <v>10</v>
       </c>
       <c r="H289">
         <v>49.656642000000012</v>
@@ -15319,7 +15322,7 @@
         <v>4.0267127999999994</v>
       </c>
       <c r="G290">
-        <v>70</v>
+        <v>10</v>
       </c>
       <c r="H290">
         <v>52.622414000000013</v>
@@ -15366,7 +15369,7 @@
         <v>1.6988144999999999</v>
       </c>
       <c r="G291">
-        <v>70</v>
+        <v>10</v>
       </c>
       <c r="H291">
         <v>55.147328000000002</v>
@@ -15413,7 +15416,7 @@
         <v>3.6850282999999999</v>
       </c>
       <c r="G292">
-        <v>70</v>
+        <v>10</v>
       </c>
       <c r="H292">
         <v>55.027094000000012</v>
@@ -15460,7 +15463,7 @@
         <v>1.8482189</v>
       </c>
       <c r="G293">
-        <v>70</v>
+        <v>10</v>
       </c>
       <c r="H293">
         <v>55.427874000000003</v>
@@ -15507,7 +15510,7 @@
         <v>1.7253566</v>
       </c>
       <c r="G294">
-        <v>70</v>
+        <v>10</v>
       </c>
       <c r="H294">
         <v>47.572586000000001</v>
@@ -15554,7 +15557,7 @@
         <v>1.5165027</v>
       </c>
       <c r="G295">
-        <v>70</v>
+        <v>10</v>
       </c>
       <c r="H295">
         <v>57.111150000000002</v>
@@ -15601,7 +15604,7 @@
         <v>1.6245927</v>
       </c>
       <c r="G296">
-        <v>70</v>
+        <v>10</v>
       </c>
       <c r="H296">
         <v>46.009544000000012</v>
@@ -15648,7 +15651,7 @@
         <v>0.8266483</v>
       </c>
       <c r="G297">
-        <v>70</v>
+        <v>10</v>
       </c>
       <c r="H297">
         <v>55.788576000000013</v>
@@ -15695,7 +15698,7 @@
         <v>0.61058840000000003</v>
       </c>
       <c r="G298">
-        <v>70</v>
+        <v>10</v>
       </c>
       <c r="H298">
         <v>51.219684000000001</v>
@@ -15742,7 +15745,7 @@
         <v>1.3699806999999999</v>
       </c>
       <c r="G299">
-        <v>70</v>
+        <v>10</v>
       </c>
       <c r="H299">
         <v>79.514752000000001</v>
@@ -15789,7 +15792,7 @@
         <v>1.0630051</v>
       </c>
       <c r="G300">
-        <v>70</v>
+        <v>10</v>
       </c>
       <c r="H300">
         <v>72.340789999999998</v>
@@ -15836,7 +15839,7 @@
         <v>0.72996780000000006</v>
       </c>
       <c r="G301">
-        <v>70</v>
+        <v>10</v>
       </c>
       <c r="H301">
         <v>50.057422000000003</v>
@@ -15883,7 +15886,7 @@
         <v>0.52567770000000003</v>
       </c>
       <c r="G302">
-        <v>70</v>
+        <v>10</v>
       </c>
       <c r="H302">
         <v>48.334068000000002</v>
@@ -15930,7 +15933,7 @@
         <v>0.7872555</v>
       </c>
       <c r="G303">
-        <v>70</v>
+        <v>10</v>
       </c>
       <c r="H303">
         <v>65.287062000000006</v>
@@ -15977,7 +15980,7 @@
         <v>0.35633670000000001</v>
       </c>
       <c r="G304">
-        <v>70</v>
+        <v>10</v>
       </c>
       <c r="H304">
         <v>46.931337999999997</v>
@@ -16024,7 +16027,7 @@
         <v>0.33279710000000001</v>
       </c>
       <c r="G305">
-        <v>70</v>
+        <v>10</v>
       </c>
       <c r="H305">
         <v>45.528608000000013</v>
@@ -16071,7 +16074,7 @@
         <v>3.3222062000000001</v>
       </c>
       <c r="G306">
-        <v>70</v>
+        <v>10</v>
       </c>
       <c r="H306">
         <v>48.774926000000001</v>
@@ -16118,7 +16121,7 @@
         <v>2.948455</v>
       </c>
       <c r="G307">
-        <v>70</v>
+        <v>10</v>
       </c>
       <c r="H307">
         <v>24.808281999999998</v>
@@ -16165,7 +16168,7 @@
         <v>0.22662869999999999</v>
       </c>
       <c r="G308">
-        <v>70</v>
+        <v>10</v>
       </c>
       <c r="H308">
         <v>35.509107999999998</v>
@@ -16212,7 +16215,7 @@
         <v>0.46742919999999999</v>
       </c>
       <c r="G309">
-        <v>70</v>
+        <v>10</v>
       </c>
       <c r="H309">
         <v>26.892337999999999</v>
@@ -16259,7 +16262,7 @@
         <v>0.85234969999999999</v>
       </c>
       <c r="G310">
-        <v>70</v>
+        <v>10</v>
       </c>
       <c r="H310">
         <v>64.966438000000011</v>
@@ -16306,7 +16309,7 @@
         <v>1.1271385</v>
       </c>
       <c r="G311">
-        <v>70</v>
+        <v>10</v>
       </c>
       <c r="H311">
         <v>38.755426</v>
@@ -16353,7 +16356,7 @@
         <v>1.4927229</v>
       </c>
       <c r="G312">
-        <v>70</v>
+        <v>10</v>
       </c>
       <c r="H312">
         <v>54.987015999999997</v>
@@ -16400,7 +16403,7 @@
         <v>0.9897440999999999</v>
       </c>
       <c r="G313">
-        <v>70</v>
+        <v>10</v>
       </c>
       <c r="H313">
         <v>57.672241999999997</v>
@@ -16447,7 +16450,7 @@
         <v>1.7409695999999999</v>
       </c>
       <c r="G314">
-        <v>70</v>
+        <v>10</v>
       </c>
       <c r="H314">
         <v>52.341868000000012</v>
@@ -16494,7 +16497,7 @@
         <v>4.4058685000000004</v>
       </c>
       <c r="G315">
-        <v>70</v>
+        <v>10</v>
       </c>
       <c r="H315">
         <v>43.604864000000013</v>
@@ -16541,7 +16544,7 @@
         <v>3.1720812</v>
       </c>
       <c r="G316">
-        <v>70</v>
+        <v>10</v>
       </c>
       <c r="H316">
         <v>47.492430000000013</v>
@@ -16588,7 +16591,7 @@
         <v>3.2228835</v>
       </c>
       <c r="G317">
-        <v>70</v>
+        <v>10</v>
       </c>
       <c r="H317">
         <v>47.612664000000002</v>
@@ -16635,7 +16638,7 @@
         <v>2.9347636000000001</v>
       </c>
       <c r="G318">
-        <v>70</v>
+        <v>10</v>
       </c>
       <c r="H318">
         <v>31.541385999999999</v>
@@ -16682,7 +16685,7 @@
         <v>3.1212789000000001</v>
       </c>
       <c r="G319">
-        <v>70</v>
+        <v>10</v>
       </c>
       <c r="H319">
         <v>45.688920000000003</v>
@@ -16729,7 +16732,7 @@
         <v>2.9763182000000001</v>
       </c>
       <c r="G320">
-        <v>70</v>
+        <v>10</v>
       </c>
       <c r="H320">
         <v>42.723148000000002</v>
@@ -16776,7 +16779,7 @@
         <v>3.2339327</v>
       </c>
       <c r="G321">
-        <v>70</v>
+        <v>10</v>
       </c>
       <c r="H321">
         <v>46.851182000000001</v>
@@ -16823,7 +16826,7 @@
         <v>2.6862767000000001</v>
       </c>
       <c r="G322">
-        <v>70</v>
+        <v>10</v>
       </c>
       <c r="H322">
         <v>32.463180000000001</v>
@@ -16870,7 +16873,7 @@
         <v>3.2477442000000001</v>
       </c>
       <c r="G323">
-        <v>70</v>
+        <v>10</v>
       </c>
       <c r="H323">
         <v>50.498280000000001</v>
@@ -16917,7 +16920,7 @@
         <v>2.2762552999999999</v>
       </c>
       <c r="G324">
-        <v>70</v>
+        <v>10</v>
       </c>
       <c r="H324">
         <v>56.750448000000013</v>
@@ -16964,7 +16967,7 @@
         <v>2.5625737000000002</v>
       </c>
       <c r="G325">
-        <v>70</v>
+        <v>10</v>
       </c>
       <c r="H325">
         <v>48.414223999999997</v>
@@ -17011,7 +17014,7 @@
         <v>1.6704709</v>
       </c>
       <c r="G326">
-        <v>70</v>
+        <v>10</v>
       </c>
       <c r="H326">
         <v>63.443474000000002</v>
@@ -17058,7 +17061,7 @@
         <v>2.1478684000000001</v>
       </c>
       <c r="G327">
-        <v>70</v>
+        <v>10</v>
       </c>
       <c r="H327">
         <v>33.905988000000001</v>
@@ -17105,7 +17108,7 @@
         <v>4.6469092000000014</v>
       </c>
       <c r="G328">
-        <v>70</v>
+        <v>10</v>
       </c>
       <c r="H328">
         <v>58.113100000000003</v>
@@ -17152,7 +17155,7 @@
         <v>1.3610933000000001</v>
       </c>
       <c r="G329">
-        <v>70</v>
+        <v>10</v>
       </c>
       <c r="H329">
         <v>63.724020000000003</v>
@@ -17199,7 +17202,7 @@
         <v>0.76924049999999999</v>
       </c>
       <c r="G330">
-        <v>70</v>
+        <v>10</v>
       </c>
       <c r="H330">
         <v>16.151433999999998</v>
@@ -17246,7 +17249,7 @@
         <v>2.8479312999999999</v>
       </c>
       <c r="G331">
-        <v>70</v>
+        <v>10</v>
       </c>
       <c r="H331">
         <v>56.389746000000002</v>
@@ -17293,7 +17296,7 @@
         <v>2.1192845999999999</v>
       </c>
       <c r="G332">
-        <v>70</v>
+        <v>10</v>
       </c>
       <c r="H332">
         <v>20.920715999999999</v>
@@ -17340,7 +17343,7 @@
         <v>1.6242323999999999</v>
       </c>
       <c r="G333">
-        <v>70</v>
+        <v>10</v>
       </c>
       <c r="H333">
         <v>35.348796</v>
@@ -17387,7 +17390,7 @@
         <v>2.2679684</v>
       </c>
       <c r="G334">
-        <v>70</v>
+        <v>10</v>
       </c>
       <c r="H334">
         <v>56.469901999999998</v>
@@ -17434,7 +17437,7 @@
         <v>2.0758084000000001</v>
       </c>
       <c r="G335">
-        <v>70</v>
+        <v>10</v>
       </c>
       <c r="H335">
         <v>64.445424000000003</v>
@@ -17481,7 +17484,7 @@
         <v>2.5182568000000001</v>
       </c>
       <c r="G336">
-        <v>70</v>
+        <v>10</v>
       </c>
       <c r="H336">
         <v>57.832554000000002</v>
@@ -17528,7 +17531,7 @@
         <v>1.9770862</v>
       </c>
       <c r="G337">
-        <v>70</v>
+        <v>10</v>
       </c>
       <c r="H337">
         <v>62.842304000000013</v>
@@ -17575,7 +17578,7 @@
         <v>1.4958454999999999</v>
       </c>
       <c r="G338">
-        <v>70</v>
+        <v>10</v>
       </c>
       <c r="H338">
         <v>59.595986000000003</v>
@@ -17622,7 +17625,7 @@
         <v>2.0462638000000002</v>
       </c>
       <c r="G339">
-        <v>70</v>
+        <v>10</v>
       </c>
       <c r="H339">
         <v>69.896032000000005</v>
@@ -17669,7 +17672,7 @@
         <v>2.2910276000000001</v>
       </c>
       <c r="G340">
-        <v>70</v>
+        <v>10</v>
       </c>
       <c r="H340">
         <v>72.74157000000001</v>
@@ -17716,7 +17719,7 @@
         <v>1.9641154000000001</v>
       </c>
       <c r="G341">
-        <v>70</v>
+        <v>10</v>
       </c>
       <c r="H341">
         <v>59.636063999999998</v>
@@ -17763,7 +17766,7 @@
         <v>1.0461910999999999</v>
       </c>
       <c r="G342">
-        <v>70</v>
+        <v>10</v>
       </c>
       <c r="H342">
         <v>51.620464000000013</v>
@@ -17810,7 +17813,7 @@
         <v>0.58392619999999995</v>
       </c>
       <c r="G343">
-        <v>70</v>
+        <v>10</v>
       </c>
       <c r="H343">
         <v>50.939138</v>
@@ -17857,7 +17860,7 @@
         <v>0.38684210000000002</v>
       </c>
       <c r="G344">
-        <v>70</v>
+        <v>10</v>
       </c>
       <c r="H344">
         <v>48.374146000000003</v>
@@ -17904,7 +17907,7 @@
         <v>1.1893503000000001</v>
       </c>
       <c r="G345">
-        <v>70</v>
+        <v>10</v>
       </c>
       <c r="H345">
         <v>52.983116000000003</v>
@@ -17951,7 +17954,7 @@
         <v>3.4306565</v>
       </c>
       <c r="G346">
-        <v>70</v>
+        <v>10</v>
       </c>
       <c r="H346">
         <v>56.30959</v>
@@ -17998,7 +18001,7 @@
         <v>4.0835200999999994</v>
       </c>
       <c r="G347">
-        <v>70</v>
+        <v>10</v>
       </c>
       <c r="H347">
         <v>55.387796000000002</v>
@@ -18045,7 +18048,7 @@
         <v>11.196442599999999</v>
       </c>
       <c r="G348">
-        <v>70</v>
+        <v>10</v>
       </c>
       <c r="H348">
         <v>38.635192000000004</v>
@@ -18092,7 +18095,7 @@
         <v>1.0138841999999999</v>
       </c>
       <c r="G349">
-        <v>70</v>
+        <v>10</v>
       </c>
       <c r="H349">
         <v>48.534458000000001</v>
@@ -18139,7 +18142,7 @@
         <v>2.4840282999999999</v>
       </c>
       <c r="G350">
-        <v>70</v>
+        <v>10</v>
       </c>
       <c r="H350">
         <v>49.616563999999997</v>
@@ -18186,7 +18189,7 @@
         <v>1.8154315999999999</v>
       </c>
       <c r="G351">
-        <v>70</v>
+        <v>10</v>
       </c>
       <c r="H351">
         <v>18.716425999999998</v>
@@ -18233,7 +18236,7 @@
         <v>2.6255061</v>
       </c>
       <c r="G352">
-        <v>70</v>
+        <v>10</v>
       </c>
       <c r="H352">
         <v>58.954738000000013</v>
@@ -18280,7 +18283,7 @@
         <v>1.6949713</v>
       </c>
       <c r="G353">
-        <v>70</v>
+        <v>10</v>
       </c>
       <c r="H353">
         <v>56.429824000000004</v>
@@ -18327,7 +18330,7 @@
         <v>1.3492033999999999</v>
       </c>
       <c r="G354">
-        <v>70</v>
+        <v>10</v>
       </c>
       <c r="H354">
         <v>31.902087999999999</v>
@@ -18374,7 +18377,7 @@
         <v>1.5626211000000001</v>
       </c>
       <c r="G355">
-        <v>70</v>
+        <v>10</v>
       </c>
       <c r="H355">
         <v>54.906860000000002</v>
@@ -18421,7 +18424,7 @@
         <v>2.8279947000000001</v>
       </c>
       <c r="G356">
-        <v>70</v>
+        <v>10</v>
       </c>
       <c r="H356">
         <v>56.590136000000001</v>
@@ -18468,7 +18471,7 @@
         <v>1.0381444</v>
       </c>
       <c r="G357">
-        <v>70</v>
+        <v>10</v>
       </c>
       <c r="H357">
         <v>36.110278000000001</v>
@@ -18515,7 +18518,7 @@
         <v>2.5899565</v>
       </c>
       <c r="G358">
-        <v>70</v>
+        <v>10</v>
       </c>
       <c r="H358">
         <v>51.941088000000001</v>
@@ -18562,7 +18565,7 @@
         <v>2.9000547000000001</v>
       </c>
       <c r="G359">
-        <v>70</v>
+        <v>10</v>
       </c>
       <c r="H359">
         <v>51.500230000000002</v>
@@ -18609,7 +18612,7 @@
         <v>2.9895292000000002</v>
       </c>
       <c r="G360">
-        <v>70</v>
+        <v>10</v>
       </c>
       <c r="H360">
         <v>50.658592000000013</v>
@@ -18656,7 +18659,7 @@
         <v>1.7989778999999999</v>
       </c>
       <c r="G361">
-        <v>70</v>
+        <v>10</v>
       </c>
       <c r="H361">
         <v>41.280340000000002</v>
@@ -18703,7 +18706,7 @@
         <v>2.2787774000000001</v>
       </c>
       <c r="G362">
-        <v>70</v>
+        <v>10</v>
       </c>
       <c r="H362">
         <v>50.217734</v>
@@ -18750,7 +18753,7 @@
         <v>0.5990588</v>
       </c>
       <c r="G363">
-        <v>70</v>
+        <v>10</v>
       </c>
       <c r="H363">
         <v>53.303739999999998</v>
@@ -18797,7 +18800,7 @@
         <v>1.0153254</v>
       </c>
       <c r="G364">
-        <v>70</v>
+        <v>10</v>
       </c>
       <c r="H364">
         <v>83.923332000000002</v>
@@ -18844,7 +18847,7 @@
         <v>0.58344580000000001</v>
       </c>
       <c r="G365">
-        <v>70</v>
+        <v>10</v>
       </c>
       <c r="H365">
         <v>48.374146000000003</v>
@@ -18891,7 +18894,7 @@
         <v>0.62151749999999995</v>
       </c>
       <c r="G366">
-        <v>70</v>
+        <v>10</v>
       </c>
       <c r="H366">
         <v>43.484630000000003</v>
@@ -18938,7 +18941,7 @@
         <v>0.50862350000000001</v>
       </c>
       <c r="G367">
-        <v>70</v>
+        <v>10</v>
       </c>
       <c r="H367">
         <v>46.851182000000001</v>
@@ -18985,7 +18988,7 @@
         <v>1.1886296999999999</v>
       </c>
       <c r="G368">
-        <v>70</v>
+        <v>10</v>
       </c>
       <c r="H368">
         <v>65.487452000000005</v>
@@ -19032,7 +19035,7 @@
         <v>0.40821990000000002</v>
       </c>
       <c r="G369">
-        <v>70</v>
+        <v>10</v>
       </c>
       <c r="H369">
         <v>42.883459999999999</v>
@@ -19079,7 +19082,7 @@
         <v>0.40305560000000001</v>
       </c>
       <c r="G370">
-        <v>70</v>
+        <v>10</v>
       </c>
       <c r="H370">
         <v>40.959716</v>
@@ -19126,7 +19129,7 @@
         <v>0.41746759999999999</v>
       </c>
       <c r="G371">
-        <v>70</v>
+        <v>10</v>
       </c>
       <c r="H371">
         <v>50.458202</v>
@@ -19173,7 +19176,7 @@
         <v>1.2916755</v>
       </c>
       <c r="G372">
-        <v>70</v>
+        <v>10</v>
       </c>
       <c r="H372">
         <v>91.417918</v>
@@ -19220,7 +19223,7 @@
         <v>0.84466330000000001</v>
       </c>
       <c r="G373">
-        <v>70</v>
+        <v>10</v>
       </c>
       <c r="H373">
         <v>41.520808000000002</v>
@@ -19267,7 +19270,7 @@
         <v>0.36702560000000001</v>
       </c>
       <c r="G374">
-        <v>70</v>
+        <v>10</v>
       </c>
       <c r="H374">
         <v>41.520808000000002</v>
@@ -19314,7 +19317,7 @@
         <v>0.92585090000000003</v>
       </c>
       <c r="G375">
-        <v>70</v>
+        <v>10</v>
       </c>
       <c r="H375">
         <v>14.468158000000001</v>
@@ -19361,7 +19364,7 @@
         <v>0.48340250000000001</v>
       </c>
       <c r="G376">
-        <v>70</v>
+        <v>10</v>
       </c>
       <c r="H376">
         <v>26.932416</v>
@@ -19408,7 +19411,7 @@
         <v>0.77308370000000004</v>
       </c>
       <c r="G377">
-        <v>70</v>
+        <v>10</v>
       </c>
       <c r="H377">
         <v>7.1739620000000004</v>
@@ -19455,7 +19458,7 @@
         <v>0.74317880000000003</v>
       </c>
       <c r="G378">
-        <v>70</v>
+        <v>10</v>
       </c>
       <c r="H378">
         <v>52.90296</v>
@@ -19502,7 +19505,7 @@
         <v>0.51510889999999998</v>
       </c>
       <c r="G379">
-        <v>70</v>
+        <v>10</v>
       </c>
       <c r="H379">
         <v>15.43003</v>
@@ -19549,7 +19552,7 @@
         <v>0.85835470000000003</v>
       </c>
       <c r="G380">
-        <v>70</v>
+        <v>10</v>
       </c>
       <c r="H380">
         <v>9.4984859999999998</v>
@@ -19596,7 +19599,7 @@
         <v>0.59953920000000005</v>
       </c>
       <c r="G381">
-        <v>70</v>
+        <v>10</v>
       </c>
       <c r="H381">
         <v>2.164212</v>
@@ -19643,7 +19646,7 @@
         <v>0.97425120000000009</v>
       </c>
       <c r="G382">
-        <v>70</v>
+        <v>10</v>
       </c>
       <c r="H382">
         <v>20.359624</v>
@@ -19690,7 +19693,7 @@
         <v>0.81643980000000005</v>
       </c>
       <c r="G383">
-        <v>70</v>
+        <v>10</v>
       </c>
       <c r="H383">
         <v>24.327345999999999</v>
@@ -19737,7 +19740,7 @@
         <v>0.80358909999999995</v>
       </c>
       <c r="G384">
-        <v>70</v>
+        <v>10</v>
       </c>
       <c r="H384">
         <v>51.780776000000003</v>
@@ -19784,7 +19787,7 @@
         <v>1.4568129999999999</v>
       </c>
       <c r="G385">
-        <v>70</v>
+        <v>10</v>
       </c>
       <c r="H385">
         <v>55.748497999999998</v>
@@ -19831,7 +19834,7 @@
         <v>1.5151816</v>
       </c>
       <c r="G386">
-        <v>70</v>
+        <v>10</v>
       </c>
       <c r="H386">
         <v>59.074972000000002</v>
@@ -19878,7 +19881,7 @@
         <v>0.97605269999999988</v>
       </c>
       <c r="G387">
-        <v>70</v>
+        <v>10</v>
       </c>
       <c r="H387">
         <v>48.774926000000001</v>

</xml_diff>